<commit_message>
Add points for cjc09ujyfc1ks4blsyl8hbfv8_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/cjc09ujyfc1ks4blsyl8hbfv8_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/cjc09ujyfc1ks4blsyl8hbfv8_playerlog.xlsx
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE2" t="n">
         <v>1</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -951,14 +951,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="AD3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE3" t="n">
         <v>1</v>
@@ -1004,21 +1004,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>-0.18249794</v>
+        <v>-0.15983657</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1134,14 +1134,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE4" t="n">
         <v>1</v>
@@ -1187,21 +1187,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>-0.12966887</v>
+        <v>-0.20716736</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1317,14 +1317,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE5" t="n">
         <v>1</v>
@@ -1370,21 +1370,21 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>-0.01381177</v>
+        <v>0.08224580000000001</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1396,10 +1396,10 @@
         <v>0</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS5" t="n">
         <v>1</v>
@@ -1439,7 +1439,7 @@
         <v>0</v>
       </c>
       <c r="BF5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG5" t="n">
         <v>0</v>
@@ -1500,14 +1500,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE6" t="n">
         <v>1</v>
@@ -1553,11 +1553,11 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.08779118999999996</v>
+        <v>0.11513916</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>-0.04</t>
         </is>
       </c>
       <c r="AK6" t="n">
@@ -1567,7 +1567,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1683,14 +1683,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="AD7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE7" t="n">
         <v>1</v>
@@ -1736,11 +1736,11 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>-0.23337663</v>
+        <v>-0.42282367</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>-0.58</t>
         </is>
       </c>
       <c r="AK7" t="n">
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS7" t="n">
         <v>0</v>
@@ -1866,14 +1866,14 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1902,7 +1902,7 @@
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE8" t="n">
         <v>1</v>
@@ -1919,24 +1919,24 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>-0.04596962</v>
+        <v>0.9740719999999999</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>-0.16</t>
+          <t>+0.82</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO8" t="n">
         <v>0</v>
@@ -1963,7 +1963,7 @@
         <v>0</v>
       </c>
       <c r="AW8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX8" t="n">
         <v>0</v>
@@ -1988,7 +1988,7 @@
         <v>0</v>
       </c>
       <c r="BF8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG8" t="n">
         <v>0</v>
@@ -2049,14 +2049,14 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="AD9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE9" t="n">
         <v>1</v>
@@ -2102,21 +2102,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>-0.12028559</v>
+        <v>0.06217640999999999</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2232,14 +2232,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2247,7 +2247,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2268,7 +2268,7 @@
         </is>
       </c>
       <c r="AD10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE10" t="n">
         <v>1</v>
@@ -2285,21 +2285,21 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.01005472</v>
+        <v>-0.01958198</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.18</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2311,7 +2311,7 @@
         <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR10" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG10" t="n">
         <v>0</v>
@@ -2415,14 +2415,14 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="AD11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE11" t="n">
         <v>1</v>
@@ -2468,21 +2468,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.005820259999999996</v>
+        <v>0.10554935</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>-0.11</t>
+          <t>-0.05</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2491,7 +2491,7 @@
         <v>0</v>
       </c>
       <c r="AP11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ11" t="n">
         <v>0</v>
@@ -2537,7 +2537,7 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG11" t="n">
         <v>0</v>
@@ -2598,14 +2598,14 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
@@ -2634,7 +2634,7 @@
         </is>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE12" t="n">
         <v>1</v>
@@ -2651,21 +2651,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>-0.21037133</v>
+        <v>-0.02464582</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>-0.32</t>
+          <t>-0.18</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2677,19 +2677,19 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS12" t="n">
         <v>0</v>
       </c>
       <c r="AT12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV12" t="n">
         <v>0</v>
@@ -2720,7 +2720,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2781,14 +2781,14 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2796,7 +2796,7 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2820,7 +2820,7 @@
         <v>1</v>
       </c>
       <c r="AE13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF13" t="n">
         <v>0</v>
@@ -2836,7 +2836,7 @@
         <v>0</v>
       </c>
       <c r="AM13" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2898,7 +2898,7 @@
         <v>0</v>
       </c>
       <c r="BG13" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14">
@@ -2956,14 +2956,14 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -2995,10 +2995,10 @@
         <v>1</v>
       </c>
       <c r="AE14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG14" t="n">
         <v>1</v>
@@ -3009,21 +3009,21 @@
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.09183689</v>
+        <v>-0.08492790000000001</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.24</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="AL14" t="n">
         <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3044,7 +3044,7 @@
         <v>0</v>
       </c>
       <c r="AT14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU14" t="n">
         <v>0</v>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="BE14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF14" t="n">
         <v>0</v>
@@ -3143,14 +3143,14 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -3182,10 +3182,10 @@
         <v>1</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG15" t="n">
         <v>1</v>
@@ -3196,21 +3196,21 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.35511422</v>
+        <v>0.2837407200000001</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>+0.24</t>
+          <t>+0.13</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL15" t="n">
         <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3219,7 +3219,7 @@
         <v>0</v>
       </c>
       <c r="AP15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ15" t="n">
         <v>0</v>
@@ -3265,7 +3265,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3326,14 +3326,14 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3365,10 +3365,10 @@
         <v>1</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG16" t="n">
         <v>1</v>
@@ -3379,21 +3379,21 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.25095129</v>
+        <v>0.20631808</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>+0.14</t>
+          <t>+0.05</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AL16" t="n">
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3509,14 +3509,14 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3548,10 +3548,10 @@
         <v>1</v>
       </c>
       <c r="AE17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG17" t="n">
         <v>1</v>
@@ -3562,21 +3562,21 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.06297892000000001</v>
+        <v>-0.16658368</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>-0.05</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="AL17" t="n">
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3638,7 +3638,7 @@
         <v>0</v>
       </c>
       <c r="BG17" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="18">
@@ -3696,14 +3696,14 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3735,10 +3735,10 @@
         <v>1</v>
       </c>
       <c r="AE18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
@@ -3749,21 +3749,21 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.07853840000000001</v>
+        <v>-0.02722645000000001</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>-0.04</t>
+          <t>-0.18</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3778,16 +3778,16 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS18" t="n">
         <v>2</v>
       </c>
       <c r="AT18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV18" t="n">
         <v>0</v>
@@ -3819,13 +3819,13 @@
         </is>
       </c>
       <c r="BE18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BF18" t="n">
         <v>0</v>
       </c>
       <c r="BG18" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19">
@@ -3883,14 +3883,14 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3922,7 +3922,7 @@
         <v>1</v>
       </c>
       <c r="AE19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF19" t="n">
         <v>0</v>
@@ -3936,21 +3936,21 @@
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.37109027</v>
+        <v>0.30560348</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>+0.26</t>
+          <t>+0.15</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -3962,10 +3962,10 @@
         <v>0</v>
       </c>
       <c r="AQ19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS19" t="n">
         <v>0</v>
@@ -3974,7 +3974,7 @@
         <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
@@ -4006,10 +4006,10 @@
         </is>
       </c>
       <c r="BE19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG19" t="n">
         <v>1</v>
@@ -4070,14 +4070,14 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4109,10 +4109,10 @@
         <v>1</v>
       </c>
       <c r="AE20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG20" t="n">
         <v>1</v>
@@ -4123,11 +4123,11 @@
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>1.54288407</v>
+        <v>1.36550291</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+1.43</t>
+          <t>+1.21</t>
         </is>
       </c>
       <c r="AK20" t="n">
@@ -4137,7 +4137,7 @@
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN20" t="n">
         <v>1</v>
@@ -4149,7 +4149,7 @@
         <v>0</v>
       </c>
       <c r="AQ20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR20" t="n">
         <v>0</v>
@@ -4192,7 +4192,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4253,14 +4253,14 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -4268,7 +4268,7 @@
         </is>
       </c>
       <c r="S21" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4292,7 +4292,7 @@
         <v>1</v>
       </c>
       <c r="AE21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF21" t="n">
         <v>0</v>
@@ -4306,11 +4306,11 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.05169223</v>
+        <v>0.06732060000000001</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="AK21" t="n">
@@ -4320,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4440,14 +4440,14 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4479,10 +4479,10 @@
         <v>1</v>
       </c>
       <c r="AE22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
@@ -4493,21 +4493,21 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.4910534</v>
+        <v>0.38290769</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.38</t>
+          <t>+0.23</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -4531,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV22" t="n">
         <v>0</v>
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="BE22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF22" t="n">
         <v>2</v>
@@ -4627,14 +4627,14 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -4642,7 +4642,7 @@
         </is>
       </c>
       <c r="S23" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4666,7 +4666,7 @@
         <v>1</v>
       </c>
       <c r="AE23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF23" t="n">
         <v>0</v>
@@ -4680,21 +4680,21 @@
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.90786134</v>
+        <v>0.9326151499999999</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>+0.79</t>
+          <t>+0.78</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>

</xml_diff>